<commit_message>
docs: added daily tracker spreadsheet
</commit_message>
<xml_diff>
--- a/backend/Backend-Dev3-Daily-Tracker.xlsx
+++ b/backend/Backend-Dev3-Daily-Tracker.xlsx
@@ -5,7 +5,7 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dell\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dell\OneDrive\Documents\Internship\Business-Listing\backend\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="33">
   <si>
     <t>40 Working Days · 8 Hours/Day · Fill in Date, Status, Hours, and Notes every day.</t>
   </si>
@@ -111,10 +111,16 @@
     <t xml:space="preserve">Backend Developer — Business Listing </t>
   </si>
   <si>
+    <t>1.  feat: draft Business, Review, Booking models with relations (pending supervisor approval)          2. docs: add ERD for Business, Review, Booking schema (pending approval)                            3. docs: mention docs/ folder in root README     4. docs: added daily tracker spreadsheet</t>
+  </si>
+  <si>
     <t>1. chore: add starter project structure (auth module implemented; listings, reviews, bookings scaffolded)
-2. chore: F11restructure repo into backend/ and frontend/ monorepo H7layout
+2. chore: F11restructure repo into backend/ and frontend/ monorepo layout
 3. chore: approve install scripts, add lockfile and initial User migration
 4. chore: switch backend port to 3001 to avoid clash with frontend default             5. Removed guideline document                          6. Deleted Backend-Dev5-Guideline.docx                 7. docs: add daily tracker spreadsheet</t>
+  </si>
+  <si>
+    <t>Drafted Business/Review/Booking schema with relations, created ERD, sent for approval                     Discussions on the project with the CEO and frontend developer to better understand the requirements      Updated Trello according to the status of the tasks</t>
   </si>
 </sst>
 </file>
@@ -207,7 +213,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -226,6 +232,9 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -575,28 +584,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="B1" s="8"/>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
-      <c r="E1" s="8"/>
-      <c r="F1" s="8"/>
-      <c r="G1" s="8"/>
-      <c r="H1" s="8"/>
+      <c r="B1" s="9"/>
+      <c r="C1" s="9"/>
+      <c r="D1" s="9"/>
+      <c r="E1" s="9"/>
+      <c r="F1" s="9"/>
+      <c r="G1" s="9"/>
+      <c r="H1" s="9"/>
     </row>
     <row r="2" spans="1:8" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="7" t="s">
+      <c r="A2" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="8"/>
-      <c r="C2" s="8"/>
-      <c r="D2" s="8"/>
-      <c r="E2" s="8"/>
-      <c r="F2" s="8"/>
-      <c r="G2" s="8"/>
-      <c r="H2" s="8"/>
+      <c r="B2" s="9"/>
+      <c r="C2" s="9"/>
+      <c r="D2" s="9"/>
+      <c r="E2" s="9"/>
+      <c r="F2" s="9"/>
+      <c r="G2" s="9"/>
+      <c r="H2" s="9"/>
     </row>
     <row r="4" spans="1:8" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
@@ -644,24 +653,32 @@
         <v>26</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="H5" s="6" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" ht="159" x14ac:dyDescent="0.3">
       <c r="A6" s="2">
         <v>2</v>
       </c>
-      <c r="B6" s="3"/>
+      <c r="B6" s="5">
+        <v>46260</v>
+      </c>
       <c r="C6" s="2"/>
-      <c r="D6" s="3"/>
+      <c r="D6" s="6" t="s">
+        <v>32</v>
+      </c>
       <c r="E6" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="F6" s="2"/>
-      <c r="G6" s="3"/>
+        <v>28</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="G6" s="7" t="s">
+        <v>30</v>
+      </c>
       <c r="H6" s="3"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.3">

</xml_diff>